<commit_message>
Add NFL International hub (/teams/nfl/international), linked from the NFL page. It leads with the modern NFL International Series: every regular-season game played outside the US since 2007, each linked to its franchises, host metro and country, with score and attendance omitted. Below sits the full NFL Europe / WLAF record (1991-2007): World Bowl champions, all sixteen franchises ranked by titles, and season standings, built from the new 'NFL Europe' sheet of OtherLeagues.xlsx into public/data/nfl/europe.json and international-series.json. The Name column is canonical, so Birmingham Fire and Rhein Fire are one club that relocated to the Rhine-Ruhr in 1995, the Scottish Claymores span Edinburgh then Glasgow, and London/England Monarchs are merged; each franchise now appears as a defunct team on its host metro pages. Page copy is kept terse with inline stat bylines.
</commit_message>
<xml_diff>
--- a/Overture-Match-Suggestions/CG.xlsx
+++ b/Overture-Match-Suggestions/CG.xlsx
@@ -1484,10 +1484,24 @@
           <t>BrazzavilleCongo</t>
         </is>
       </c>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>CG-BZV</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Brazzaville (département)</t>
+        </is>
+      </c>
       <c r="Q12" s="3" t="n"/>
       <c r="R12" s="3" t="n"/>
       <c r="S12" s="3" t="n"/>
@@ -4594,10 +4608,24 @@
           <t>NiariCongo</t>
         </is>
       </c>
-      <c r="M48" s="2" t="n"/>
-      <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="n"/>
-      <c r="P48" s="2" t="n"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>county</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>CG-11</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>Louvakou (Loubomo)</t>
+        </is>
+      </c>
       <c r="Q48" s="2" t="n"/>
       <c r="R48" s="2" t="n"/>
       <c r="S48" s="2" t="n"/>
@@ -6712,10 +6740,24 @@
           <t>Pointe-NoireCongo</t>
         </is>
       </c>
-      <c r="M73" s="3" t="n"/>
-      <c r="N73" s="3" t="n"/>
-      <c r="O73" s="3" t="n"/>
-      <c r="P73" s="3" t="n"/>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>county</t>
+        </is>
+      </c>
+      <c r="N73" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O73" s="3" t="inlineStr">
+        <is>
+          <t>CG-8</t>
+        </is>
+      </c>
+      <c r="P73" s="3" t="inlineStr">
+        <is>
+          <t>Loandjili (Pointe Noire)</t>
+        </is>
+      </c>
       <c r="Q73" s="3" t="n"/>
       <c r="R73" s="3" t="n"/>
       <c r="S73" s="3" t="n"/>
@@ -6900,10 +6942,24 @@
           <t>PoolCongo</t>
         </is>
       </c>
-      <c r="M75" s="2" t="n"/>
-      <c r="N75" s="2" t="n"/>
-      <c r="O75" s="2" t="n"/>
-      <c r="P75" s="2" t="n"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>CG-BZV</t>
+        </is>
+      </c>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>Brazzaville (département)</t>
+        </is>
+      </c>
       <c r="Q75" s="2" t="n"/>
       <c r="R75" s="2" t="n"/>
       <c r="S75" s="2" t="n"/>

</xml_diff>